<commit_message>
Update ACT table through WK2635
</commit_message>
<xml_diff>
--- a/ACT table.xlsx
+++ b/ACT table.xlsx
@@ -6712,7 +6712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ49"/>
+  <dimension ref="A1:AL49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
@@ -6902,6 +6902,16 @@
           <t>W2633</t>
         </is>
       </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>W2634</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>W2635</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -7001,6 +7011,12 @@
       <c r="AJ2" s="3" t="n">
         <v>4005</v>
       </c>
+      <c r="AK2" s="3" t="n">
+        <v>4355</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>4679</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -7142,6 +7158,12 @@
       <c r="AJ4" s="3" t="n">
         <v>6711</v>
       </c>
+      <c r="AK4" s="3" t="n">
+        <v>7163</v>
+      </c>
+      <c r="AL4" s="3" t="n">
+        <v>7578</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -7214,6 +7236,12 @@
       <c r="AJ5" s="3" t="n">
         <v>3327</v>
       </c>
+      <c r="AK5" s="3" t="n">
+        <v>3678</v>
+      </c>
+      <c r="AL5" s="3" t="n">
+        <v>4009</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -7553,6 +7581,12 @@
       <c r="AJ12" s="3" t="n">
         <v>10289</v>
       </c>
+      <c r="AK12" s="3" t="n">
+        <v>12090</v>
+      </c>
+      <c r="AL12" s="3" t="n">
+        <v>13127</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -7613,6 +7647,12 @@
       <c r="AJ13" s="3" t="n">
         <v>100121</v>
       </c>
+      <c r="AK13" s="3" t="n">
+        <v>110638</v>
+      </c>
+      <c r="AL13" s="3" t="n">
+        <v>119760</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -7673,6 +7713,12 @@
       <c r="AJ14" s="3" t="n">
         <v>18137</v>
       </c>
+      <c r="AK14" s="3" t="n">
+        <v>19630</v>
+      </c>
+      <c r="AL14" s="3" t="n">
+        <v>20767</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -7733,6 +7779,12 @@
       <c r="AJ15" s="3" t="n">
         <v>522</v>
       </c>
+      <c r="AK15" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="AL15" s="3" t="n">
+        <v>669</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -7793,6 +7845,12 @@
       <c r="AJ16" s="3" t="n">
         <v>923</v>
       </c>
+      <c r="AK16" s="3" t="n">
+        <v>1138</v>
+      </c>
+      <c r="AL16" s="3" t="n">
+        <v>1350</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -7850,6 +7908,12 @@
       <c r="AJ17" s="3" t="n">
         <v>884</v>
       </c>
+      <c r="AK17" s="3" t="n">
+        <v>1003</v>
+      </c>
+      <c r="AL17" s="3" t="n">
+        <v>1110</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -7910,6 +7974,12 @@
       <c r="AJ18" s="3" t="n">
         <v>1034</v>
       </c>
+      <c r="AK18" s="3" t="n">
+        <v>1153</v>
+      </c>
+      <c r="AL18" s="3" t="n">
+        <v>1279</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -8021,6 +8091,12 @@
       <c r="AJ20" s="3" t="n">
         <v>161</v>
       </c>
+      <c r="AK20" s="3" t="n">
+        <v>170</v>
+      </c>
+      <c r="AL20" s="3" t="n">
+        <v>181</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -8132,6 +8208,12 @@
       <c r="AJ22" s="3" t="n">
         <v>459</v>
       </c>
+      <c r="AK22" s="3" t="n">
+        <v>532</v>
+      </c>
+      <c r="AL22" s="3" t="n">
+        <v>608</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -8192,6 +8274,12 @@
       <c r="AJ23" s="3" t="n">
         <v>870</v>
       </c>
+      <c r="AK23" s="3" t="n">
+        <v>978</v>
+      </c>
+      <c r="AL23" s="3" t="n">
+        <v>1062</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -8252,6 +8340,12 @@
       <c r="AJ24" s="3" t="n">
         <v>1947</v>
       </c>
+      <c r="AK24" s="3" t="n">
+        <v>2134</v>
+      </c>
+      <c r="AL24" s="3" t="n">
+        <v>2320</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -8312,6 +8406,12 @@
       <c r="AJ25" s="3" t="n">
         <v>538</v>
       </c>
+      <c r="AK25" s="3" t="n">
+        <v>590</v>
+      </c>
+      <c r="AL25" s="3" t="n">
+        <v>656</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -8372,6 +8472,12 @@
       <c r="AJ26" s="3" t="n">
         <v>1081</v>
       </c>
+      <c r="AK26" s="3" t="n">
+        <v>1220</v>
+      </c>
+      <c r="AL26" s="3" t="n">
+        <v>1350</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -8432,6 +8538,12 @@
       <c r="AJ27" s="3" t="n">
         <v>1646</v>
       </c>
+      <c r="AK27" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="AL27" s="3" t="n">
+        <v>2058</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -8492,6 +8604,12 @@
       <c r="AJ28" s="3" t="n">
         <v>661</v>
       </c>
+      <c r="AK28" s="3" t="n">
+        <v>711</v>
+      </c>
+      <c r="AL28" s="3" t="n">
+        <v>772</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -8552,6 +8670,12 @@
       <c r="AJ29" s="3" t="n">
         <v>1742</v>
       </c>
+      <c r="AK29" s="3" t="n">
+        <v>1832</v>
+      </c>
+      <c r="AL29" s="3" t="n">
+        <v>1905</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -8630,6 +8754,12 @@
       <c r="AJ30" s="3" t="n">
         <v>2441</v>
       </c>
+      <c r="AK30" s="3" t="n">
+        <v>2512</v>
+      </c>
+      <c r="AL30" s="3" t="n">
+        <v>2574</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -8933,6 +9063,12 @@
       <c r="AJ35" s="3" t="n">
         <v>6384</v>
       </c>
+      <c r="AK35" s="3" t="n">
+        <v>6690</v>
+      </c>
+      <c r="AL35" s="3" t="n">
+        <v>7018</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -8993,6 +9129,12 @@
       <c r="AJ36" s="3" t="n">
         <v>650</v>
       </c>
+      <c r="AK36" s="3" t="n">
+        <v>706</v>
+      </c>
+      <c r="AL36" s="3" t="n">
+        <v>780</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -9053,6 +9195,12 @@
       <c r="AJ37" s="3" t="n">
         <v>902</v>
       </c>
+      <c r="AK37" s="3" t="n">
+        <v>1017</v>
+      </c>
+      <c r="AL37" s="3" t="n">
+        <v>1176</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -9116,6 +9264,12 @@
       <c r="AJ38" s="3" t="n">
         <v>3350</v>
       </c>
+      <c r="AK38" s="3" t="n">
+        <v>3646</v>
+      </c>
+      <c r="AL38" s="3" t="n">
+        <v>3956</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -9215,6 +9369,12 @@
       <c r="AJ39" s="3" t="n">
         <v>8647</v>
       </c>
+      <c r="AK39" s="3" t="n">
+        <v>9227</v>
+      </c>
+      <c r="AL39" s="3" t="n">
+        <v>9778</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -9314,6 +9474,12 @@
       <c r="AJ40" s="3" t="n">
         <v>3066</v>
       </c>
+      <c r="AK40" s="3" t="n">
+        <v>3525</v>
+      </c>
+      <c r="AL40" s="3" t="n">
+        <v>3929</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -9380,6 +9546,12 @@
       <c r="AJ41" s="3" t="n">
         <v>6616</v>
       </c>
+      <c r="AK41" s="3" t="n">
+        <v>7400</v>
+      </c>
+      <c r="AL41" s="3" t="n">
+        <v>8135</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -9632,6 +9804,12 @@
       <c r="AJ45" s="3" t="n">
         <v>11120</v>
       </c>
+      <c r="AK45" s="3" t="n">
+        <v>11880</v>
+      </c>
+      <c r="AL45" s="3" t="n">
+        <v>12623</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -9692,6 +9870,12 @@
       <c r="AJ46" s="3" t="n">
         <v>1727</v>
       </c>
+      <c r="AK46" s="3" t="n">
+        <v>1852</v>
+      </c>
+      <c r="AL46" s="3" t="n">
+        <v>1985</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -9752,6 +9936,12 @@
       <c r="AJ47" s="3" t="n">
         <v>3103</v>
       </c>
+      <c r="AK47" s="3" t="n">
+        <v>3287</v>
+      </c>
+      <c r="AL47" s="3" t="n">
+        <v>3466</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -9812,6 +10002,12 @@
       <c r="AJ48" s="3" t="n">
         <v>1392</v>
       </c>
+      <c r="AK48" s="3" t="n">
+        <v>1540</v>
+      </c>
+      <c r="AL48" s="3" t="n">
+        <v>1782</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -9910,6 +10106,12 @@
       </c>
       <c r="AJ49" s="3" t="n">
         <v>8345</v>
+      </c>
+      <c r="AK49" s="3" t="n">
+        <v>9074</v>
+      </c>
+      <c r="AL49" s="3" t="n">
+        <v>9680</v>
       </c>
     </row>
   </sheetData>

</xml_diff>